<commit_message>
renamed cruise 1 files and modified .xlsx file.
</commit_message>
<xml_diff>
--- a/SSD-Metadata.xlsx
+++ b/SSD-Metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uncw4-my.sharepoint.com/personal/dem5075_uncw_edu/Documents/SSD/src/Jupyter_Notebook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uncw4-my.sharepoint.com/personal/dem5075_uncw_edu/Documents/SSD/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="275" documentId="8_{40F56BEC-5573-1D48-86DD-62B78177A085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B59B3E11-B4DE-5848-89FE-0F0C3AECA13E}"/>
+  <xr:revisionPtr revIDLastSave="454" documentId="8_{40F56BEC-5573-1D48-86DD-62B78177A085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88DE9A7B-2525-604C-ACA6-EEFB868978E0}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="620" windowWidth="34420" windowHeight="28180" xr2:uid="{06BCB4AE-F001-1547-BAA2-CC230ADAC34F}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="15140" windowHeight="18960" xr2:uid="{06BCB4AE-F001-1547-BAA2-CC230ADAC34F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="114">
   <si>
     <t>Date</t>
   </si>
@@ -134,10 +134,253 @@
     <t>Cloudy</t>
   </si>
   <si>
-    <t>Cast went under boat.</t>
-  </si>
-  <si>
     <t>Start_time</t>
+  </si>
+  <si>
+    <t>kjdabv</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>260527-01(NC11)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-02(ACME)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-03(DP)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-04(BBT)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-05(IC-1)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-05(IC-2)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-06(NAV)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-07(HB)-A016.txt</t>
+  </si>
+  <si>
+    <t>260527-08(NCF6)-A016.txt</t>
+  </si>
+  <si>
+    <t>260603-01(NCF6)-A016.txt</t>
+  </si>
+  <si>
+    <t>260603-02(NC11)-A016.txt</t>
+  </si>
+  <si>
+    <t>260603-03(ACME)-A016.txt</t>
+  </si>
+  <si>
+    <t>260603-04(DP)-A016.txt</t>
+  </si>
+  <si>
+    <t>260603-05(BBT)-A016.txt</t>
+  </si>
+  <si>
+    <t>260603-06(IC)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-01(M18)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-02(M23)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-03(M35)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-04(M54)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-05(BRR)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-06(NAV)-A016.txt</t>
+  </si>
+  <si>
+    <t>260610-07(HB)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-01(NC11)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-01(NC11)-A017.txt</t>
+  </si>
+  <si>
+    <t>260618-02(ACME)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-02(ACME)-A017.txt</t>
+  </si>
+  <si>
+    <t>260618-03(DP)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-03(DP)-A017.txt</t>
+  </si>
+  <si>
+    <t>260618-04(BBT)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-04(BBT)-A017.txt</t>
+  </si>
+  <si>
+    <t>260618-05(IC)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-05(IC)-A017.txt</t>
+  </si>
+  <si>
+    <t>260618-06(NCF6)-A016.txt</t>
+  </si>
+  <si>
+    <t>260618-06(NCF6)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-01(M18)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-01(M18)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-02(M23)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-03(M35)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-04(M54)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-05(BRR)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-06(M61)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-07(HB)-A017.txt</t>
+  </si>
+  <si>
+    <t>260625-08(NAV)-A017.txt</t>
+  </si>
+  <si>
+    <t>IC-1</t>
+  </si>
+  <si>
+    <t>IC-2</t>
+  </si>
+  <si>
+    <t>260702-02(M23-1)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-02(M23-2)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-03(M35)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-04(M54)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-05(BRR)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-05(M61)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-07(HB)-A017.txt</t>
+  </si>
+  <si>
+    <t>260702-08(NAV)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-01(NCF6)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-02(NC11)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-03(ACME)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-04(DP)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-05(BBT-1)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-05(BBT-2)-A017.txt</t>
+  </si>
+  <si>
+    <t>260709-06(IC)-A017.txt</t>
+  </si>
+  <si>
+    <t>260716-01(M18)-A017-txt</t>
+  </si>
+  <si>
+    <t>260716-02(M23)-A017-txt</t>
+  </si>
+  <si>
+    <t>260716-03(M35)-A017-txt</t>
+  </si>
+  <si>
+    <t>260716-04(M54)-A017-txt</t>
+  </si>
+  <si>
+    <t>260716-05(BRR)-A017-txt</t>
+  </si>
+  <si>
+    <t>260716-06(M61)-A017-txt</t>
+  </si>
+  <si>
+    <t>260716-07(NCF6)-A017-txt</t>
+  </si>
+  <si>
+    <t>ACME-1</t>
+  </si>
+  <si>
+    <t>ACME-2</t>
+  </si>
+  <si>
+    <t>NAV-1</t>
+  </si>
+  <si>
+    <t>NAV-2</t>
+  </si>
+  <si>
+    <t>270728-01(NC11)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-02(ACME-1)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-02(ACME-2)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-03(DP)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-04(BBT)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-05(IC)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-06(NAV-1)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-01(NAV-2)-A017.txt</t>
+  </si>
+  <si>
+    <t>270728-07(HB)-A017.txt</t>
   </si>
 </sst>
 </file>
@@ -197,6 +440,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -516,17 +763,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82548158-EA7E-374B-ADC5-7AD11079E1E4}">
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="7" max="7" width="73.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.1640625" customWidth="1"/>
+    <col min="7" max="7" width="13.1640625" customWidth="1"/>
+    <col min="8" max="8" width="65.1640625" customWidth="1"/>
     <col min="9" max="9" width="15.1640625" customWidth="1"/>
     <col min="10" max="10" width="14.6640625" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -534,1178 +783,1568 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>26</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>27</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>28</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>260527</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="1">
         <v>0.65695601851851848</v>
       </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
         <v>260527</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="1">
         <v>0.67743055555555554</v>
       </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>260527</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="1">
         <v>0.69480324074074074</v>
       </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5">
         <v>260527</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="1">
         <v>0.7005555555555556</v>
       </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
         <v>260527</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="1">
         <v>0.711400462962963</v>
       </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7">
         <v>260527</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="1">
         <v>0.7173032407407407</v>
       </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8">
         <v>260527</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="1">
         <v>0.72777777777777775</v>
       </c>
-      <c r="D8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9">
         <v>260527</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1">
         <v>0.74340277777777775</v>
       </c>
-      <c r="D9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10">
         <v>260527</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="1">
         <v>0.75646990740740738</v>
       </c>
-      <c r="D10" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2</v>
       </c>
       <c r="B11">
         <v>260603</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="1">
         <v>0.63402777777777775</v>
       </c>
-      <c r="D11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2</v>
       </c>
       <c r="B12">
         <v>260603</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="1">
         <v>0.69849537037037035</v>
       </c>
-      <c r="D12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2</v>
       </c>
       <c r="B13">
         <v>260603</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="1">
         <v>0.71862268518518524</v>
       </c>
-      <c r="D13" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2</v>
       </c>
       <c r="B14">
         <v>260603</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="1">
         <v>0.7368055555555556</v>
       </c>
-      <c r="D14" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2</v>
       </c>
       <c r="B15">
         <v>260603</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="1">
         <v>0.74856481481481485</v>
       </c>
-      <c r="D15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16">
         <v>260603</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="1">
         <v>0.76249999999999996</v>
       </c>
-      <c r="D16" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>3</v>
       </c>
       <c r="B17">
         <v>260610</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="1">
         <v>0.63638888888888889</v>
       </c>
-      <c r="D17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>3</v>
       </c>
       <c r="B18">
         <v>260610</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="1">
         <v>0.6489583333333333</v>
       </c>
-      <c r="D18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>3</v>
       </c>
       <c r="B19">
         <v>260610</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="1">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D19" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>3</v>
       </c>
       <c r="B20">
         <v>260610</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="1">
         <v>0.68181712962962959</v>
       </c>
-      <c r="D20" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>3</v>
       </c>
       <c r="B21">
         <v>260610</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="1">
         <v>0.69680555555555557</v>
       </c>
-      <c r="D21" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>3</v>
       </c>
       <c r="B22">
         <v>260610</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="1">
         <v>0.75416666666666665</v>
       </c>
-      <c r="D22" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>3</v>
       </c>
       <c r="B23">
         <v>260610</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" t="s">
+        <v>55</v>
+      </c>
+      <c r="F23" s="1">
         <v>0.76410879629629624</v>
       </c>
-      <c r="D23" t="s">
-        <v>6</v>
-      </c>
-      <c r="E23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>4</v>
       </c>
       <c r="B24">
         <v>260618</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" s="1">
         <v>0.64326388888888886</v>
       </c>
-      <c r="D24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E24" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>4</v>
       </c>
       <c r="B25">
         <v>260618</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="1">
         <v>0.64758101851851857</v>
       </c>
-      <c r="D25" t="s">
-        <v>7</v>
-      </c>
-      <c r="E25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>4</v>
       </c>
       <c r="B26">
         <v>260618</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="1">
         <v>0.66138888888888892</v>
       </c>
-      <c r="D26" t="s">
-        <v>6</v>
-      </c>
-      <c r="E26" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>4</v>
       </c>
       <c r="B27">
         <v>260618</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F27" s="1">
         <v>0.66488425925925931</v>
       </c>
-      <c r="D27" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4</v>
       </c>
       <c r="B28">
         <v>260618</v>
       </c>
-      <c r="C28" s="1">
+      <c r="C28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" t="s">
+        <v>6</v>
+      </c>
+      <c r="E28" t="s">
+        <v>60</v>
+      </c>
+      <c r="F28" s="1">
         <v>0.6802083333333333</v>
       </c>
-      <c r="D28" t="s">
-        <v>6</v>
-      </c>
-      <c r="E28" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4</v>
       </c>
       <c r="B29">
         <v>260618</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" t="s">
+        <v>61</v>
+      </c>
+      <c r="F29" s="1">
         <v>0.6850694444444444</v>
       </c>
-      <c r="D29" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4</v>
       </c>
       <c r="B30">
         <v>260618</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" t="s">
+        <v>62</v>
+      </c>
+      <c r="F30" s="1">
         <v>0.69515046296296301</v>
       </c>
-      <c r="D30" t="s">
-        <v>6</v>
-      </c>
-      <c r="E30" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4</v>
       </c>
       <c r="B31">
         <v>260618</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" t="s">
+        <v>63</v>
+      </c>
+      <c r="F31" s="1">
         <v>0.70021990740740736</v>
       </c>
-      <c r="D31" t="s">
-        <v>7</v>
-      </c>
-      <c r="E31" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4</v>
       </c>
       <c r="B32">
         <v>260618</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32" t="s">
+        <v>64</v>
+      </c>
+      <c r="F32" s="1">
         <v>0.71250000000000002</v>
       </c>
-      <c r="D32" t="s">
-        <v>6</v>
-      </c>
-      <c r="E32" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4</v>
       </c>
       <c r="B33">
         <v>260618</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" t="s">
+        <v>65</v>
+      </c>
+      <c r="F33" s="1">
         <v>0.71792824074074069</v>
       </c>
-      <c r="D33" t="s">
-        <v>7</v>
-      </c>
-      <c r="E33" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4</v>
       </c>
       <c r="B34">
         <v>260618</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34" t="s">
+        <v>66</v>
+      </c>
+      <c r="F34" s="1">
         <v>0.74652777777777779</v>
       </c>
-      <c r="D34" t="s">
-        <v>6</v>
-      </c>
-      <c r="E34" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4</v>
       </c>
       <c r="B35">
         <v>260618</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" t="s">
+        <v>67</v>
+      </c>
+      <c r="F35" s="1">
         <v>0.75124999999999997</v>
       </c>
-      <c r="D35" t="s">
-        <v>7</v>
-      </c>
-      <c r="E35" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>5</v>
       </c>
       <c r="B36">
         <v>260625</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C36" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+      <c r="E36" t="s">
+        <v>68</v>
+      </c>
+      <c r="F36" s="1">
         <v>0.63056712962962957</v>
       </c>
-      <c r="D36" t="s">
-        <v>7</v>
-      </c>
-      <c r="E36" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>5</v>
       </c>
       <c r="B37">
         <v>260625</v>
       </c>
-      <c r="C37" s="1">
+      <c r="C37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" t="s">
+        <v>7</v>
+      </c>
+      <c r="E37" t="s">
+        <v>70</v>
+      </c>
+      <c r="F37" s="1">
         <v>0.70451388888888888</v>
       </c>
-      <c r="D37" t="s">
-        <v>7</v>
-      </c>
-      <c r="E37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>5</v>
       </c>
       <c r="B38">
         <v>260625</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C38" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" t="s">
+        <v>7</v>
+      </c>
+      <c r="E38" t="s">
+        <v>71</v>
+      </c>
+      <c r="F38" s="1">
         <v>0.72291666666666665</v>
       </c>
-      <c r="D38" t="s">
-        <v>7</v>
-      </c>
-      <c r="E38" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>5</v>
       </c>
       <c r="B39">
         <v>260625</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" t="s">
+        <v>7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>72</v>
+      </c>
+      <c r="F39" s="1">
         <v>0.74291666666666667</v>
       </c>
-      <c r="D39" t="s">
-        <v>7</v>
-      </c>
-      <c r="E39" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>5</v>
       </c>
       <c r="B40">
         <v>260625</v>
       </c>
-      <c r="C40" s="1">
+      <c r="C40" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" t="s">
+        <v>73</v>
+      </c>
+      <c r="F40" s="1">
         <v>0.76076388888888891</v>
       </c>
-      <c r="D40" t="s">
-        <v>7</v>
-      </c>
-      <c r="E40" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>5</v>
       </c>
       <c r="B41">
         <v>260625</v>
       </c>
-      <c r="C41" s="1">
+      <c r="C41" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" t="s">
+        <v>7</v>
+      </c>
+      <c r="E41" t="s">
+        <v>74</v>
+      </c>
+      <c r="F41" s="1">
         <v>0.77487268518518515</v>
       </c>
-      <c r="D41" t="s">
-        <v>7</v>
-      </c>
-      <c r="E41" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>5</v>
       </c>
       <c r="B42">
         <v>260625</v>
       </c>
-      <c r="C42" s="1">
+      <c r="C42" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" s="1">
         <v>0.79237268518518522</v>
       </c>
-      <c r="D42" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>5</v>
       </c>
       <c r="B43">
         <v>260625</v>
       </c>
-      <c r="C43" s="1">
+      <c r="C43" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" t="s">
+        <v>76</v>
+      </c>
+      <c r="F43" s="1">
         <v>0.8052083333333333</v>
       </c>
-      <c r="D43" t="s">
-        <v>7</v>
-      </c>
-      <c r="E43" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>6</v>
       </c>
       <c r="B44">
         <v>260702</v>
       </c>
-      <c r="C44" s="1">
+      <c r="C44" t="s">
+        <v>16</v>
+      </c>
+      <c r="D44" t="s">
+        <v>7</v>
+      </c>
+      <c r="E44" t="s">
+        <v>69</v>
+      </c>
+      <c r="F44" s="1">
         <v>0.62765046296296301</v>
       </c>
-      <c r="D44" t="s">
-        <v>7</v>
-      </c>
-      <c r="E44" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>6</v>
       </c>
       <c r="B45">
         <v>260702</v>
       </c>
-      <c r="C45" s="1">
+      <c r="C45" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45" t="s">
+        <v>7</v>
+      </c>
+      <c r="E45" t="s">
+        <v>79</v>
+      </c>
+      <c r="F45" s="1">
         <v>0.63888888888888884</v>
       </c>
-      <c r="D45" t="s">
-        <v>7</v>
-      </c>
-      <c r="E45" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>6</v>
       </c>
       <c r="B46">
         <v>260702</v>
       </c>
-      <c r="C46" s="1">
+      <c r="C46" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" t="s">
+        <v>7</v>
+      </c>
+      <c r="E46" t="s">
+        <v>80</v>
+      </c>
+      <c r="F46" s="1">
         <v>0.6430555555555556</v>
       </c>
-      <c r="D46" t="s">
-        <v>7</v>
-      </c>
-      <c r="E46" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>6</v>
       </c>
       <c r="B47">
         <v>260702</v>
       </c>
-      <c r="C47" s="1">
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" t="s">
+        <v>7</v>
+      </c>
+      <c r="E47" t="s">
+        <v>81</v>
+      </c>
+      <c r="F47" s="1">
         <v>0.6538194444444444</v>
       </c>
-      <c r="D47" t="s">
-        <v>7</v>
-      </c>
-      <c r="E47" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>6</v>
       </c>
       <c r="B48">
         <v>260702</v>
       </c>
-      <c r="C48" s="1">
+      <c r="C48" t="s">
+        <v>19</v>
+      </c>
+      <c r="D48" t="s">
+        <v>7</v>
+      </c>
+      <c r="E48" t="s">
+        <v>82</v>
+      </c>
+      <c r="F48" s="1">
         <v>0.67146990740740742</v>
       </c>
-      <c r="D48" t="s">
-        <v>7</v>
-      </c>
-      <c r="E48" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>6</v>
       </c>
       <c r="B49">
         <v>260702</v>
       </c>
-      <c r="C49" s="1">
+      <c r="C49" t="s">
+        <v>20</v>
+      </c>
+      <c r="D49" t="s">
+        <v>7</v>
+      </c>
+      <c r="E49" t="s">
+        <v>83</v>
+      </c>
+      <c r="F49" s="1">
         <v>0.68501157407407409</v>
       </c>
-      <c r="D49" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>6</v>
       </c>
       <c r="B50">
         <v>260702</v>
       </c>
-      <c r="C50" s="1">
+      <c r="C50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" t="s">
+        <v>7</v>
+      </c>
+      <c r="E50" t="s">
+        <v>84</v>
+      </c>
+      <c r="F50" s="1">
         <v>0.72710648148148149</v>
       </c>
-      <c r="D50" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>6</v>
       </c>
       <c r="B51">
         <v>260702</v>
       </c>
-      <c r="C51" s="1">
+      <c r="C51" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" t="s">
+        <v>85</v>
+      </c>
+      <c r="F51" s="1">
         <v>0.74056712962962967</v>
       </c>
-      <c r="D51" t="s">
-        <v>7</v>
-      </c>
-      <c r="E51" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>6</v>
       </c>
       <c r="B52">
         <v>260702</v>
       </c>
-      <c r="C52" s="1">
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" t="s">
+        <v>7</v>
+      </c>
+      <c r="E52" t="s">
+        <v>86</v>
+      </c>
+      <c r="F52" s="1">
         <v>0.74646990740740737</v>
       </c>
-      <c r="D52" t="s">
-        <v>7</v>
-      </c>
-      <c r="E52" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>7</v>
       </c>
       <c r="B53">
         <v>260709</v>
       </c>
-      <c r="C53" s="1">
+      <c r="C53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D53" t="s">
+        <v>7</v>
+      </c>
+      <c r="E53" t="s">
+        <v>87</v>
+      </c>
+      <c r="F53" s="1">
         <v>0.63431712962962961</v>
       </c>
-      <c r="D53" t="s">
-        <v>7</v>
-      </c>
-      <c r="E53" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>7</v>
       </c>
       <c r="B54">
         <v>260709</v>
       </c>
-      <c r="C54" s="1">
+      <c r="C54" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" t="s">
+        <v>7</v>
+      </c>
+      <c r="E54" t="s">
+        <v>88</v>
+      </c>
+      <c r="F54" s="1">
         <v>0.68256944444444445</v>
       </c>
-      <c r="D54" t="s">
-        <v>7</v>
-      </c>
-      <c r="E54" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>7</v>
       </c>
       <c r="B55">
         <v>260709</v>
       </c>
-      <c r="C55" s="1">
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
+        <v>7</v>
+      </c>
+      <c r="E55" t="s">
+        <v>89</v>
+      </c>
+      <c r="F55" s="1">
         <v>0.70402777777777781</v>
       </c>
-      <c r="D55" t="s">
-        <v>7</v>
-      </c>
-      <c r="E55" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>7</v>
       </c>
       <c r="B56">
         <v>260709</v>
       </c>
-      <c r="C56" s="1">
+      <c r="C56" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" t="s">
+        <v>7</v>
+      </c>
+      <c r="E56" t="s">
+        <v>90</v>
+      </c>
+      <c r="F56" s="1">
         <v>0.72048611111111116</v>
       </c>
-      <c r="D56" t="s">
-        <v>7</v>
-      </c>
-      <c r="E56" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>7</v>
       </c>
       <c r="B57">
         <v>260709</v>
       </c>
-      <c r="C57" s="1">
+      <c r="C57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D57" t="s">
+        <v>7</v>
+      </c>
+      <c r="E57" t="s">
+        <v>91</v>
+      </c>
+      <c r="F57" s="1">
         <v>0.72916666666666663</v>
       </c>
-      <c r="D57" t="s">
-        <v>7</v>
-      </c>
-      <c r="E57" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>7</v>
       </c>
       <c r="B58">
         <v>260709</v>
       </c>
-      <c r="C58" s="1">
+      <c r="C58" t="s">
+        <v>25</v>
+      </c>
+      <c r="D58" t="s">
+        <v>7</v>
+      </c>
+      <c r="E58" t="s">
+        <v>92</v>
+      </c>
+      <c r="F58" s="1">
         <v>0.7318055555555556</v>
       </c>
-      <c r="D58" t="s">
-        <v>7</v>
-      </c>
-      <c r="E58" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>7</v>
       </c>
       <c r="B59">
         <v>260709</v>
       </c>
-      <c r="C59" s="1">
+      <c r="C59" t="s">
+        <v>12</v>
+      </c>
+      <c r="D59" t="s">
+        <v>7</v>
+      </c>
+      <c r="E59" t="s">
+        <v>93</v>
+      </c>
+      <c r="F59" s="1">
         <v>0.74481481481481482</v>
       </c>
-      <c r="D59" t="s">
-        <v>7</v>
-      </c>
-      <c r="E59" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>8</v>
       </c>
       <c r="B60">
         <v>260716</v>
       </c>
-      <c r="C60" s="1">
+      <c r="C60" t="s">
+        <v>16</v>
+      </c>
+      <c r="D60" t="s">
+        <v>7</v>
+      </c>
+      <c r="E60" t="s">
+        <v>94</v>
+      </c>
+      <c r="F60" s="1">
         <v>0.63320601851851854</v>
       </c>
-      <c r="D60" t="s">
-        <v>7</v>
-      </c>
-      <c r="E60" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>8</v>
       </c>
       <c r="B61">
         <v>260716</v>
       </c>
-      <c r="C61" s="1">
+      <c r="C61" t="s">
+        <v>17</v>
+      </c>
+      <c r="D61" t="s">
+        <v>7</v>
+      </c>
+      <c r="E61" t="s">
+        <v>95</v>
+      </c>
+      <c r="F61" s="1">
         <v>0.64430555555555558</v>
       </c>
-      <c r="D61" t="s">
-        <v>7</v>
-      </c>
-      <c r="E61" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>8</v>
       </c>
       <c r="B62">
         <v>260716</v>
       </c>
-      <c r="C62" s="1">
+      <c r="C62" t="s">
+        <v>18</v>
+      </c>
+      <c r="D62" t="s">
+        <v>7</v>
+      </c>
+      <c r="E62" t="s">
+        <v>96</v>
+      </c>
+      <c r="F62" s="1">
         <v>0.65972222222222221</v>
       </c>
-      <c r="D62" t="s">
-        <v>7</v>
-      </c>
-      <c r="E62" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>8</v>
       </c>
       <c r="B63">
         <v>260716</v>
       </c>
-      <c r="C63" s="1">
+      <c r="C63" t="s">
+        <v>19</v>
+      </c>
+      <c r="D63" t="s">
+        <v>7</v>
+      </c>
+      <c r="E63" t="s">
+        <v>97</v>
+      </c>
+      <c r="F63" s="1">
         <v>0.67487268518518517</v>
       </c>
-      <c r="D63" t="s">
-        <v>7</v>
-      </c>
-      <c r="E63" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>8</v>
       </c>
       <c r="B64">
         <v>260716</v>
       </c>
-      <c r="C64" s="1">
+      <c r="C64" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64" t="s">
+        <v>7</v>
+      </c>
+      <c r="E64" t="s">
+        <v>98</v>
+      </c>
+      <c r="F64" s="1">
         <v>0.70340277777777782</v>
       </c>
-      <c r="D64" t="s">
-        <v>7</v>
-      </c>
-      <c r="E64" t="s">
-        <v>20</v>
-      </c>
-      <c r="H64" s="1">
+      <c r="I64" s="1">
         <v>0.70412037037037034</v>
       </c>
-      <c r="I64" s="1">
+      <c r="J64" s="1">
         <v>0.70436342592592593</v>
       </c>
-      <c r="J64" s="1">
+      <c r="K64" s="1">
         <v>0.70458333333333334</v>
       </c>
-      <c r="K64" s="1">
+      <c r="L64" s="1">
         <v>0.7051736111111111</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>8</v>
       </c>
       <c r="B65">
         <v>260716</v>
       </c>
-      <c r="C65" s="1">
+      <c r="C65" t="s">
+        <v>21</v>
+      </c>
+      <c r="D65" t="s">
+        <v>7</v>
+      </c>
+      <c r="E65" t="s">
+        <v>99</v>
+      </c>
+      <c r="F65" s="1">
         <v>0.71416666666666662</v>
       </c>
-      <c r="D65" t="s">
-        <v>7</v>
-      </c>
-      <c r="E65" t="s">
-        <v>21</v>
-      </c>
-      <c r="H65" s="1">
+      <c r="I65" s="1">
         <v>0.71445601851851848</v>
       </c>
-      <c r="I65" s="1">
+      <c r="J65" s="1">
         <v>0.71524305555555556</v>
       </c>
-      <c r="J65" s="1">
+      <c r="K65" s="1">
         <v>0.71681712962962962</v>
       </c>
-      <c r="K65" s="1">
+      <c r="L65" s="1">
         <v>0.7174652777777778</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="N65" s="1">
+        <v>0.71524305555555556</v>
+      </c>
+      <c r="O65" s="1">
+        <v>0.71681712962962962</v>
+      </c>
+      <c r="P65" s="1">
+        <v>0.7155555555555555</v>
+      </c>
+      <c r="Q65" s="1">
+        <v>0.71649305555555554</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>8</v>
       </c>
       <c r="B66">
         <v>260716</v>
       </c>
-      <c r="C66" s="1">
+      <c r="C66" t="s">
+        <v>15</v>
+      </c>
+      <c r="D66" t="s">
+        <v>7</v>
+      </c>
+      <c r="E66" t="s">
+        <v>100</v>
+      </c>
+      <c r="F66" s="1">
         <v>0.73368055555555556</v>
       </c>
-      <c r="D66" t="s">
-        <v>7</v>
-      </c>
-      <c r="E66" t="s">
-        <v>15</v>
-      </c>
-      <c r="F66" t="s">
+      <c r="G66" t="s">
         <v>30</v>
       </c>
-      <c r="G66" t="s">
-        <v>31</v>
-      </c>
-      <c r="H66" s="1">
+      <c r="H66" t="s">
+        <v>32</v>
+      </c>
+      <c r="I66" s="1">
         <v>0.73429398148148151</v>
       </c>
-      <c r="I66" s="1">
+      <c r="J66" s="1">
         <v>0.7349768518518518</v>
       </c>
-      <c r="J66" s="1">
+      <c r="K66" s="1">
         <v>0.73511574074074071</v>
       </c>
-      <c r="K66" s="1">
+      <c r="L66" s="1">
         <v>0.7356018518518519</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>9</v>
+      </c>
+      <c r="B67">
+        <v>270728</v>
+      </c>
+      <c r="C67" t="s">
+        <v>8</v>
+      </c>
+      <c r="D67" t="s">
+        <v>7</v>
+      </c>
+      <c r="E67" t="s">
+        <v>105</v>
+      </c>
+      <c r="F67" s="1">
+        <v>0.66041666666666665</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>9</v>
+      </c>
+      <c r="B68">
+        <v>270728</v>
+      </c>
+      <c r="C68" t="s">
+        <v>101</v>
+      </c>
+      <c r="D68" t="s">
+        <v>7</v>
+      </c>
+      <c r="E68" t="s">
+        <v>106</v>
+      </c>
+      <c r="F68" s="1">
+        <v>0.67500000000000004</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>9</v>
+      </c>
+      <c r="B69">
+        <v>270728</v>
+      </c>
+      <c r="C69" t="s">
+        <v>102</v>
+      </c>
+      <c r="D69" t="s">
+        <v>7</v>
+      </c>
+      <c r="E69" t="s">
+        <v>107</v>
+      </c>
+      <c r="F69" s="1">
+        <v>0.67848379629629629</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>9</v>
+      </c>
+      <c r="B70">
+        <v>270728</v>
+      </c>
+      <c r="C70" t="s">
+        <v>10</v>
+      </c>
+      <c r="D70" t="s">
+        <v>7</v>
+      </c>
+      <c r="E70" t="s">
+        <v>108</v>
+      </c>
+      <c r="F70" s="1">
+        <v>0.69160879629629635</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>9</v>
+      </c>
+      <c r="B71">
+        <v>270728</v>
+      </c>
+      <c r="C71" t="s">
+        <v>11</v>
+      </c>
+      <c r="D71" t="s">
+        <v>7</v>
+      </c>
+      <c r="E71" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71" s="1">
+        <v>0.69958333333333333</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>9</v>
+      </c>
+      <c r="B72">
+        <v>270728</v>
+      </c>
+      <c r="C72" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" t="s">
+        <v>7</v>
+      </c>
+      <c r="E72" t="s">
+        <v>110</v>
+      </c>
+      <c r="F72" s="1">
+        <v>0.71666666666666667</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>9</v>
+      </c>
+      <c r="B73">
+        <v>270728</v>
+      </c>
+      <c r="C73" t="s">
+        <v>103</v>
+      </c>
+      <c r="D73" t="s">
+        <v>7</v>
+      </c>
+      <c r="E73" t="s">
+        <v>111</v>
+      </c>
+      <c r="F73" s="1">
+        <v>0.72881944444444446</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>9</v>
+      </c>
+      <c r="B74">
+        <v>270728</v>
+      </c>
+      <c r="C74" t="s">
+        <v>104</v>
+      </c>
+      <c r="D74" t="s">
+        <v>7</v>
+      </c>
+      <c r="E74" t="s">
+        <v>112</v>
+      </c>
+      <c r="F74" s="1">
+        <v>0.73291666666666666</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>9</v>
+      </c>
+      <c r="B75">
+        <v>270728</v>
+      </c>
+      <c r="C75" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" t="s">
+        <v>7</v>
+      </c>
+      <c r="E75" t="s">
+        <v>113</v>
+      </c>
+      <c r="F75" s="1">
+        <v>0.74091435185185184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished updating SSD-metadata, KD-Conversion updated and now reflects KD calculated from windowss, figures generated for each cast.
</commit_message>
<xml_diff>
--- a/SSD-Metadata.xlsx
+++ b/SSD-Metadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uncw4-my.sharepoint.com/personal/dem5075_uncw_edu/Documents/SSD/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1451" documentId="8_{40F56BEC-5573-1D48-86DD-62B78177A085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01F68A99-A5B8-F443-9299-B30D980512CC}"/>
+  <xr:revisionPtr revIDLastSave="1715" documentId="8_{40F56BEC-5573-1D48-86DD-62B78177A085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60F78146-F0D5-0046-8107-3FA45B4F51DE}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{06BCB4AE-F001-1547-BAA2-CC230ADAC34F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="265">
   <si>
     <t>Date</t>
   </si>
@@ -309,9 +309,6 @@
     <t>260728-06(NAV-1)-A017.txt</t>
   </si>
   <si>
-    <t>260728-01(NAV-2)-A017.txt</t>
-  </si>
-  <si>
     <t>260728-07(HB)-A017.txt</t>
   </si>
   <si>
@@ -363,9 +360,6 @@
     <t>260811-02(NC11)-A017.txt</t>
   </si>
   <si>
-    <t>260811-04(DP)-A017.txt</t>
-  </si>
-  <si>
     <t>260811-06(IC)-A016.txt</t>
   </si>
   <si>
@@ -393,9 +387,6 @@
     <t>260814-07(NCF6)-A016.txt</t>
   </si>
   <si>
-    <t>Start idx up was changed to add 2 sec to account for 10 second interval</t>
-  </si>
-  <si>
     <t>KD suffers.</t>
   </si>
   <si>
@@ -543,9 +534,6 @@
     <t xml:space="preserve">Sunny. </t>
   </si>
   <si>
-    <t xml:space="preserve">Depth: unknown;  line: unknown. </t>
-  </si>
-  <si>
     <t>Depth: 4.2m; line: unknown.</t>
   </si>
   <si>
@@ -657,9 +645,6 @@
     <t>Depth: 4.5m; line: 8.2m.</t>
   </si>
   <si>
-    <t>h</t>
-  </si>
-  <si>
     <t>Depth: 5.9m; line: 8.0m.</t>
   </si>
   <si>
@@ -687,9 +672,6 @@
     <t>Depth: 7.4m; line: 15.0m. Downcast was not smooth, only upcast has usable data.</t>
   </si>
   <si>
-    <t>Depth: 7.1m; line 10.5m. Downcast was not smooth, only upcast has usable data.</t>
-  </si>
-  <si>
     <t>260618-02(ACME-1)-A016.txt</t>
   </si>
   <si>
@@ -756,12 +738,6 @@
     <t xml:space="preserve">Depth: 4.2m; line: 5.2m. Shadow from caster affecting cast. </t>
   </si>
   <si>
-    <t>Depth: 3.9m; line: 8.5m. SSD bobs in and out of shady area. SSD handle slipping from sweaty hands. SSD passed under boat near end of cast.</t>
-  </si>
-  <si>
-    <t>Depth: 6.7m; line: 12.0m. Hiccup at 6m, line felt loose at 11.5m mark, SsD may have hit bottom. SSD went under tree during last 6m of upcast.</t>
-  </si>
-  <si>
     <t>Depth: 5.3m; line: 10.0m. Boat drifted close to shore.</t>
   </si>
   <si>
@@ -790,6 +766,75 @@
   </si>
   <si>
     <t>Depth: 15.3m; line: 10.0m. Choppy conditions.</t>
+  </si>
+  <si>
+    <t>Depth: 7.1m; line: 10.5m. Downcast was not smooth, only upcast has usable data.</t>
+  </si>
+  <si>
+    <t>Cloudy and raining.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth: unknown; line: unknown. </t>
+  </si>
+  <si>
+    <t>Depth: 9.2m; line: 20.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 6.1m; line: 16.6m.</t>
+  </si>
+  <si>
+    <t>Depth: 5.1m; line: 20.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 7.5m; line: 20.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 4.4m; line: 6.6m.</t>
+  </si>
+  <si>
+    <t>Depth: 6.0m; line: 6.9m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth: 8.9m; line: 10.6m. Heavy rain the day prior/overnight. </t>
+  </si>
+  <si>
+    <t>Depth: 13.0m; line: 10.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 10.1m; line: 10.0m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth: 5.0m; line: 10.0m. </t>
+  </si>
+  <si>
+    <t>Depth: 4.9m; line: 7.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 14.0m; line: 10.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 11.7m; line: 10.0m.</t>
+  </si>
+  <si>
+    <t>Depth: 14.1m; line: 10.0m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth: 11.3m; line: 10.0m. </t>
+  </si>
+  <si>
+    <t>260728-06(NAV-2)-A017.txt</t>
+  </si>
+  <si>
+    <t>Depth: 3.9m; line: 8.5m. SSD bobs in and out of shady area. SSD handle slipping from sweaty hands. SSD passed under boat near end of cast. SSD turned off mid-cast.</t>
+  </si>
+  <si>
+    <t>Upcast contains only 6 valid data points.</t>
+  </si>
+  <si>
+    <t>Upcast contains only 8 valid data points.</t>
+  </si>
+  <si>
+    <t>SSD shut off mid-cast; no upcast interval.</t>
   </si>
 </sst>
 </file>
@@ -1179,7 +1224,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82548158-EA7E-374B-ADC5-7AD11079E1E4}">
-  <dimension ref="A1:S104"/>
+  <dimension ref="A1:S103"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -1222,7 +1267,7 @@
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>25</v>
@@ -1237,16 +1282,16 @@
         <v>28</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="O1" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -1269,10 +1314,10 @@
         <v>0.65695601851851848</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I2" s="2">
         <v>0.65793981481481478</v>
@@ -1307,10 +1352,10 @@
         <v>0.67743055555555554</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I3" s="2">
         <v>0.67805555555555552</v>
@@ -1345,10 +1390,10 @@
         <v>0.69480324074074074</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I4" s="2">
         <v>0.69562500000000005</v>
@@ -1383,10 +1428,10 @@
         <v>0.7005555555555556</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I5" s="2">
         <v>0.7013194444444445</v>
@@ -1421,10 +1466,10 @@
         <v>0.711400462962963</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I6" s="2">
         <v>0.71211805555555552</v>
@@ -1459,10 +1504,10 @@
         <v>0.7173032407407407</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I7" s="2">
         <v>0.71800925925925929</v>
@@ -1497,10 +1542,10 @@
         <v>0.72777777777777775</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I8" s="2">
         <v>0.72843749999999996</v>
@@ -1535,10 +1580,10 @@
         <v>0.74340277777777775</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I9" s="2">
         <v>0.74422453703703706</v>
@@ -1573,10 +1618,10 @@
         <v>0.75646990740740738</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I10" s="2">
         <v>0.75725694444444447</v>
@@ -1611,10 +1656,10 @@
         <v>0.63402777777777775</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="I11" s="2">
         <v>0.63487268518518514</v>
@@ -1649,10 +1694,10 @@
         <v>0.69849537037037035</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I12" s="2">
         <v>0.69916666666666671</v>
@@ -1687,10 +1732,10 @@
         <v>0.71862268518518524</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I13" s="2">
         <v>0.7194328703703704</v>
@@ -1725,10 +1770,10 @@
         <v>0.7368055555555556</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="I14" s="2">
         <v>0.73752314814814812</v>
@@ -1763,10 +1808,10 @@
         <v>0.74856481481481485</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I15" s="2">
         <v>0.74932870370370375</v>
@@ -1801,10 +1846,10 @@
         <v>0.76249999999999996</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="I16" s="2">
         <v>0.7630555555555556</v>
@@ -1839,10 +1884,10 @@
         <v>0.63638888888888889</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I17" s="2">
         <v>0.63777777777777778</v>
@@ -1877,10 +1922,10 @@
         <v>0.6489583333333333</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I18" s="2">
         <v>0.65001157407407406</v>
@@ -1915,10 +1960,10 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="I19" s="2">
         <v>0.66773148148148154</v>
@@ -1953,10 +1998,10 @@
         <v>0.68181712962962959</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I20" s="2">
         <v>0.68246527777777777</v>
@@ -1991,10 +2036,10 @@
         <v>0.69680555555555557</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I21" s="2">
         <v>0.69730324074074079</v>
@@ -2029,10 +2074,10 @@
         <v>0.75416666666666665</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I22" s="2">
         <v>0.75434027777777779</v>
@@ -2067,10 +2112,10 @@
         <v>0.76410879629629624</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="I23" s="2">
         <v>0.76471064814814815</v>
@@ -2099,22 +2144,22 @@
         <v>260618</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="F24" s="2">
         <v>0.64326388888888886</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I24" s="2">
         <v>0.64385416666666662</v>
@@ -2137,22 +2182,22 @@
         <v>260618</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="F25" s="2">
         <v>0.64758101851851857</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="I25" s="2">
         <v>0.64820601851851856</v>
@@ -2181,16 +2226,16 @@
         <v>5</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="F26" s="2">
         <v>0.66138888888888892</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="I26" s="2">
         <v>0.66190972222222222</v>
@@ -2219,16 +2264,16 @@
         <v>6</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="F27" s="2">
         <v>0.66488425925925931</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I27" s="2">
         <v>0.66535879629629635</v>
@@ -2251,22 +2296,22 @@
         <v>260618</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="F28" s="2">
         <v>0.6802083333333333</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="I28" s="2">
         <v>0.68050925925925931</v>
@@ -2289,22 +2334,22 @@
         <v>260618</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="F29" s="2">
         <v>0.6850694444444444</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I29" s="2">
         <v>0.68555555555555558</v>
@@ -2333,16 +2378,16 @@
         <v>5</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="F30" s="2">
         <v>0.69515046296296301</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I30" s="2">
         <v>0.69574074074074077</v>
@@ -2371,16 +2416,16 @@
         <v>6</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F31" s="2">
         <v>0.70021990740740736</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="I31" s="2">
         <v>0.70048611111111114</v>
@@ -2409,16 +2454,16 @@
         <v>5</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="F32" s="2">
         <v>0.71250000000000002</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I32" s="2">
         <v>0.71302083333333333</v>
@@ -2447,16 +2492,16 @@
         <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="F33" s="2">
         <v>0.71792824074074069</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I33" s="2">
         <v>0.71836805555555561</v>
@@ -2465,13 +2510,13 @@
         <v>0.71862268518518524</v>
       </c>
       <c r="K33" s="2">
-        <v>0.71966435185185185</v>
+        <v>0.71957175925925931</v>
       </c>
       <c r="L33" s="2">
         <v>0.71966435185185185</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>117</v>
+        <v>263</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
@@ -2482,22 +2527,22 @@
         <v>260618</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="F34" s="2">
         <v>0.74652777777777779</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I34" s="2">
         <v>0.74687499999999996</v>
@@ -2520,22 +2565,22 @@
         <v>260618</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="F35" s="2">
         <v>0.75124999999999997</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I35" s="2">
         <v>0.75211805555555555</v>
@@ -2570,10 +2615,10 @@
         <v>0.63056712962962957</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="I36" s="2">
         <v>0.63140046296296293</v>
@@ -2588,7 +2633,7 @@
         <v>0.63320601851851854</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.2">
@@ -2611,10 +2656,10 @@
         <v>0.70451388888888888</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I37" s="2">
         <v>0.70512731481481483</v>
@@ -2649,10 +2694,10 @@
         <v>0.72291666666666665</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I38" s="2">
         <v>0.72331018518518519</v>
@@ -2667,7 +2712,7 @@
         <v>0.72675925925925922</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="P38" s="2">
         <v>0.72291666666666665</v>
@@ -2702,10 +2747,10 @@
         <v>0.74291666666666667</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I39" s="2">
         <v>0.74353009259259262</v>
@@ -2740,10 +2785,10 @@
         <v>0.76076388888888891</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I40" s="2">
         <v>0.76116898148148149</v>
@@ -2778,10 +2823,10 @@
         <v>0.77487268518518515</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I41" s="2">
         <v>0.77534722222222219</v>
@@ -2816,10 +2861,10 @@
         <v>0.79237268518518522</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I42" s="2">
         <v>0.79280092592592588</v>
@@ -2854,10 +2899,10 @@
         <v>0.8052083333333333</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="I43" s="2">
         <v>0.80568287037037034</v>
@@ -2892,10 +2937,10 @@
         <v>0.62765046296296301</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I44" s="2">
         <v>0.62812500000000004</v>
@@ -2930,10 +2975,10 @@
         <v>0.63888888888888884</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="I45" s="2">
         <v>0.63937500000000003</v>
@@ -2968,10 +3013,10 @@
         <v>0.6430555555555556</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="I46" s="2">
         <v>0.6434375</v>
@@ -3006,10 +3051,10 @@
         <v>0.6538194444444444</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I47" s="2">
         <v>0.61285879629629625</v>
@@ -3044,10 +3089,10 @@
         <v>0.67146990740740742</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="I48" s="2">
         <v>0.67193287037037042</v>
@@ -3082,10 +3127,10 @@
         <v>0.68501157407407409</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="I49" s="2">
         <v>0.68557870370370366</v>
@@ -3114,16 +3159,16 @@
         <v>6</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F50" s="2">
         <v>0.72710648148148149</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>167</v>
+        <v>244</v>
       </c>
       <c r="I50" s="2">
         <v>0.72774305555555552</v>
@@ -3158,10 +3203,10 @@
         <v>0.74056712962962967</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="I51" s="2">
         <v>0.74098379629629629</v>
@@ -3196,10 +3241,10 @@
         <v>0.74646990740740737</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="I52" s="2">
         <v>0.74695601851851856</v>
@@ -3234,10 +3279,10 @@
         <v>0.63431712962962961</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="I53" s="2">
         <v>0.63468749999999996</v>
@@ -3272,10 +3317,10 @@
         <v>0.68256944444444445</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I54" s="2">
         <v>0.68321759259259263</v>
@@ -3310,10 +3355,10 @@
         <v>0.70402777777777781</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="I55" s="2">
         <v>0.70468750000000002</v>
@@ -3348,10 +3393,10 @@
         <v>0.72048611111111116</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="I56" s="2">
         <v>0.72090277777777778</v>
@@ -3386,10 +3431,10 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="I57" s="2">
         <v>0.7299768518518519</v>
@@ -3424,10 +3469,10 @@
         <v>0.7318055555555556</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I58" s="2">
         <v>0.73203703703703704</v>
@@ -3462,10 +3507,10 @@
         <v>0.74481481481481482</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="I59" s="2">
         <v>0.74518518518518517</v>
@@ -3494,19 +3539,28 @@
         <v>6</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F60" s="2">
         <v>0.63320601851851854</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="I60" s="1" t="s">
-        <v>205</v>
+        <v>233</v>
+      </c>
+      <c r="I60" s="2">
+        <v>0.63396990740740744</v>
+      </c>
+      <c r="J60" s="2">
+        <v>0.63535879629629632</v>
+      </c>
+      <c r="K60" s="2">
+        <v>0.63537037037037036</v>
+      </c>
+      <c r="L60" s="2">
+        <v>0.63680555555555551</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
@@ -3523,19 +3577,28 @@
         <v>6</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F61" s="2">
         <v>0.64430555555555558</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="I61" s="1" t="s">
-        <v>205</v>
+        <v>170</v>
+      </c>
+      <c r="I61" s="2">
+        <v>0.64493055555555556</v>
+      </c>
+      <c r="J61" s="2">
+        <v>0.6464699074074074</v>
+      </c>
+      <c r="K61" s="2">
+        <v>0.64648148148148143</v>
+      </c>
+      <c r="L61" s="2">
+        <v>0.64833333333333332</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
@@ -3552,19 +3615,28 @@
         <v>6</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F62" s="2">
         <v>0.65972222222222221</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>205</v>
+        <v>171</v>
+      </c>
+      <c r="I62" s="2">
+        <v>0.66037037037037039</v>
+      </c>
+      <c r="J62" s="2">
+        <v>0.66174768518518523</v>
+      </c>
+      <c r="K62" s="2">
+        <v>0.66175925925925927</v>
+      </c>
+      <c r="L62" s="2">
+        <v>0.66355324074074074</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
@@ -3581,19 +3653,28 @@
         <v>6</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F63" s="2">
         <v>0.67487268518518517</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="I63" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
+      </c>
+      <c r="I63" s="2">
+        <v>0.67531249999999998</v>
+      </c>
+      <c r="J63" s="2">
+        <v>0.67561342592592588</v>
+      </c>
+      <c r="K63" s="2">
+        <v>0.67781250000000004</v>
+      </c>
+      <c r="L63" s="2">
+        <v>0.67803240740740744</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
@@ -3610,16 +3691,16 @@
         <v>6</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F64" s="2">
         <v>0.70340277777777782</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I64" s="2">
         <v>0.70412037037037034</v>
@@ -3648,16 +3729,16 @@
         <v>6</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F65" s="2">
         <v>0.71416666666666662</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="I65" s="2">
         <v>0.71445601851851848</v>
@@ -3698,16 +3779,16 @@
         <v>6</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F66" s="2">
         <v>0.73368055555555556</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="I66" s="2">
         <v>0.73429398148148151</v>
@@ -3742,13 +3823,22 @@
         <v>0.66041666666666665</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
+      </c>
+      <c r="I67" s="2">
+        <v>0.66107638888888887</v>
+      </c>
+      <c r="J67" s="2">
+        <v>0.66130787037037042</v>
+      </c>
+      <c r="K67" s="2">
+        <v>0.66223379629629631</v>
+      </c>
+      <c r="L67" s="2">
+        <v>0.66251157407407413</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.2">
@@ -3771,13 +3861,22 @@
         <v>0.67500000000000004</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="I68" s="1" t="s">
         <v>205</v>
+      </c>
+      <c r="I68" s="2">
+        <v>0.67552083333333335</v>
+      </c>
+      <c r="J68" s="2">
+        <v>0.67609953703703707</v>
+      </c>
+      <c r="K68" s="2">
+        <v>0.6766550925925926</v>
+      </c>
+      <c r="L68" s="2">
+        <v>0.67710648148148145</v>
       </c>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.2">
@@ -3800,13 +3899,22 @@
         <v>0.67848379629629629</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="I69" s="1" t="s">
-        <v>205</v>
+        <v>199</v>
+      </c>
+      <c r="I69" s="2">
+        <v>0.67874999999999996</v>
+      </c>
+      <c r="J69" s="2">
+        <v>0.67921296296296296</v>
+      </c>
+      <c r="K69" s="2">
+        <v>0.67943287037037037</v>
+      </c>
+      <c r="L69" s="2">
+        <v>0.67994212962962963</v>
       </c>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.2">
@@ -3829,13 +3937,22 @@
         <v>0.69160879629629635</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
+      </c>
+      <c r="I70" s="2">
+        <v>0.69209490740740742</v>
+      </c>
+      <c r="J70" s="2">
+        <v>0.69246527777777778</v>
+      </c>
+      <c r="K70" s="2">
+        <v>0.69348379629629631</v>
+      </c>
+      <c r="L70" s="2">
+        <v>0.69446759259259261</v>
       </c>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.2">
@@ -3858,13 +3975,22 @@
         <v>0.69958333333333333</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="I71" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
+      </c>
+      <c r="I71" s="2">
+        <v>0.70034722222222223</v>
+      </c>
+      <c r="J71" s="2">
+        <v>0.70075231481481481</v>
+      </c>
+      <c r="K71" s="2">
+        <v>0.70144675925925926</v>
+      </c>
+      <c r="L71" s="2">
+        <v>0.70188657407407407</v>
       </c>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.2">
@@ -3887,13 +4013,22 @@
         <v>0.71666666666666667</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="I72" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
+      </c>
+      <c r="I72" s="2">
+        <v>0.71715277777777775</v>
+      </c>
+      <c r="J72" s="2">
+        <v>0.7174652777777778</v>
+      </c>
+      <c r="K72" s="2">
+        <v>0.71859953703703705</v>
+      </c>
+      <c r="L72" s="2">
+        <v>0.71878472222222223</v>
       </c>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.2">
@@ -3916,13 +4051,22 @@
         <v>0.72881944444444446</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
+      </c>
+      <c r="I73" s="2">
+        <v>0.72917824074074078</v>
+      </c>
+      <c r="J73" s="2">
+        <v>0.72930555555555554</v>
+      </c>
+      <c r="K73" s="2">
+        <v>0.73059027777777774</v>
+      </c>
+      <c r="L73" s="2">
+        <v>0.73084490740740737</v>
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.2">
@@ -3939,19 +4083,31 @@
         <v>6</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>89</v>
+        <v>260</v>
       </c>
       <c r="F74" s="2">
         <v>0.73291666666666666</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="I74" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
+      </c>
+      <c r="I74" s="2">
+        <v>0.73348379629629634</v>
+      </c>
+      <c r="J74" s="2">
+        <v>0.73371527777777779</v>
+      </c>
+      <c r="K74" s="2">
+        <v>0.73564814814814816</v>
+      </c>
+      <c r="L74" s="2">
+        <v>0.73570601851851847</v>
+      </c>
+      <c r="O74" s="1" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.2">
@@ -3968,19 +4124,28 @@
         <v>6</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F75" s="2">
         <v>0.74091435185185184</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="I75" s="1" t="s">
-        <v>205</v>
+        <v>242</v>
+      </c>
+      <c r="I75" s="2">
+        <v>0.74131944444444442</v>
+      </c>
+      <c r="J75" s="2">
+        <v>0.74140046296296291</v>
+      </c>
+      <c r="K75" s="2">
+        <v>0.74334490740740744</v>
+      </c>
+      <c r="L75" s="2">
+        <v>0.74351851851851847</v>
       </c>
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.2">
@@ -3997,13 +4162,28 @@
         <v>6</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F76" s="2">
         <v>0.62848379629629625</v>
       </c>
-      <c r="I76" s="1" t="s">
-        <v>205</v>
+      <c r="G76" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="I76" s="2">
+        <v>0.62880787037037034</v>
+      </c>
+      <c r="J76" s="2">
+        <v>0.62935185185185183</v>
+      </c>
+      <c r="K76" s="2">
+        <v>0.62936342592592598</v>
+      </c>
+      <c r="L76" s="2">
+        <v>0.62965277777777773</v>
       </c>
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.2">
@@ -4020,13 +4200,28 @@
         <v>6</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F77" s="2">
         <v>0.63716435185185183</v>
       </c>
-      <c r="I77" s="1" t="s">
-        <v>205</v>
+      <c r="G77" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="I77" s="2">
+        <v>0.63829861111111108</v>
+      </c>
+      <c r="J77" s="2">
+        <v>0.63885416666666661</v>
+      </c>
+      <c r="K77" s="2">
+        <v>0.63923611111111112</v>
+      </c>
+      <c r="L77" s="2">
+        <v>0.63968749999999996</v>
       </c>
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.2">
@@ -4043,13 +4238,28 @@
         <v>6</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F78" s="2">
         <v>0.64881944444444439</v>
       </c>
-      <c r="I78" s="1" t="s">
-        <v>205</v>
+      <c r="G78" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="I78" s="2">
+        <v>0.64973379629629635</v>
+      </c>
+      <c r="J78" s="2">
+        <v>0.65065972222222224</v>
+      </c>
+      <c r="K78" s="2">
+        <v>0.65106481481481482</v>
+      </c>
+      <c r="L78" s="2">
+        <v>0.65127314814814818</v>
       </c>
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.2">
@@ -4066,13 +4276,28 @@
         <v>6</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F79" s="2">
         <v>0.66416666666666668</v>
       </c>
-      <c r="I79" s="1" t="s">
-        <v>205</v>
+      <c r="G79" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="I79" s="2">
+        <v>0.66532407407407412</v>
+      </c>
+      <c r="J79" s="2">
+        <v>0.66592592592592592</v>
+      </c>
+      <c r="K79" s="2">
+        <v>0.66608796296296291</v>
+      </c>
+      <c r="L79" s="2">
+        <v>0.6666319444444444</v>
       </c>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.2">
@@ -4089,16 +4314,31 @@
         <v>6</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F80" s="2">
         <v>0.67798611111111107</v>
       </c>
-      <c r="I80" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G80" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I80" s="2">
+        <v>0.67839120370370365</v>
+      </c>
+      <c r="J80" s="2">
+        <v>0.67869212962962966</v>
+      </c>
+      <c r="K80" s="2">
+        <v>0.67906250000000001</v>
+      </c>
+      <c r="L80" s="2">
+        <v>0.67925925925925923</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>10</v>
       </c>
@@ -4112,16 +4352,31 @@
         <v>6</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F81" s="2">
         <v>0.69219907407407411</v>
       </c>
-      <c r="I81" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G81" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="I81" s="2">
+        <v>0.69321759259259264</v>
+      </c>
+      <c r="J81" s="2">
+        <v>0.69344907407407408</v>
+      </c>
+      <c r="K81" s="2">
+        <v>0.69346064814814812</v>
+      </c>
+      <c r="L81" s="2">
+        <v>0.69363425925925926</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>10</v>
       </c>
@@ -4135,16 +4390,31 @@
         <v>6</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F82" s="2">
         <v>0.69473379629629628</v>
       </c>
-      <c r="I82" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G82" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="I82" s="2">
+        <v>0.69662037037037039</v>
+      </c>
+      <c r="J82" s="2">
+        <v>0.69671296296296292</v>
+      </c>
+      <c r="K82" s="2">
+        <v>0.69775462962962964</v>
+      </c>
+      <c r="L82" s="2">
+        <v>0.69785879629629632</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>10</v>
       </c>
@@ -4158,16 +4428,32 @@
         <v>6</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F83" s="2">
         <v>0.70446759259259262</v>
       </c>
-      <c r="I83" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G83" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="I83" s="2">
+        <v>0.70611111111111113</v>
+      </c>
+      <c r="J83" s="2">
+        <v>0.70640046296296299</v>
+      </c>
+      <c r="K83" s="2">
+        <v>0.70703703703703702</v>
+      </c>
+      <c r="L83" s="2">
+        <v>0.70730324074074069</v>
+      </c>
+      <c r="Q83" s="2"/>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>10</v>
       </c>
@@ -4181,16 +4467,31 @@
         <v>6</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F84" s="2">
         <v>0.71972222222222226</v>
       </c>
-      <c r="I84" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G84" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I84" s="2">
+        <v>0.72057870370370369</v>
+      </c>
+      <c r="J84" s="2">
+        <v>0.72092592592592597</v>
+      </c>
+      <c r="K84" s="2">
+        <v>0.72152777777777777</v>
+      </c>
+      <c r="L84" s="2">
+        <v>0.72189814814814812</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>11</v>
       </c>
@@ -4204,22 +4505,31 @@
         <v>6</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F85" s="2">
         <v>0.65451388888888884</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="I85" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+      <c r="I85" s="2">
+        <v>0.65511574074074075</v>
+      </c>
+      <c r="J85" s="2">
+        <v>0.65553240740740737</v>
+      </c>
+      <c r="K85" s="2">
+        <v>0.65724537037037034</v>
+      </c>
+      <c r="L85" s="2">
+        <v>0.65775462962962961</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>11</v>
       </c>
@@ -4233,22 +4543,31 @@
         <v>6</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F86" s="2">
         <v>0.70972222222222225</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="I86" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+      <c r="I86" s="2">
+        <v>0.71026620370370375</v>
+      </c>
+      <c r="J86" s="2">
+        <v>0.7106365740740741</v>
+      </c>
+      <c r="K86" s="2">
+        <v>0.71106481481481476</v>
+      </c>
+      <c r="L86" s="2">
+        <v>0.71136574074074077</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>11</v>
       </c>
@@ -4262,22 +4581,28 @@
         <v>6</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="F87" s="2">
         <v>0.72657407407407404</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="I87" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+      <c r="I87" s="2">
+        <v>0.7270833333333333</v>
+      </c>
+      <c r="J87" s="2">
+        <v>0.7275462962962963</v>
+      </c>
+      <c r="O87" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>11</v>
       </c>
@@ -4285,28 +4610,37 @@
         <v>260811</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>107</v>
       </c>
       <c r="F88" s="2">
-        <v>0.75923611111111111</v>
+        <v>0.77534722222222219</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="I88" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+        <v>234</v>
+      </c>
+      <c r="I88" s="2">
+        <v>0.77574074074074073</v>
+      </c>
+      <c r="J88" s="2">
+        <v>0.77608796296296301</v>
+      </c>
+      <c r="K88" s="2">
+        <v>0.77802083333333338</v>
+      </c>
+      <c r="L88" s="2">
+        <v>0.77813657407407411</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>11</v>
       </c>
@@ -4314,36 +4648,45 @@
         <v>260811</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D89" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F89" s="2">
-        <v>0.77534722222222219</v>
+        <v>0.78597222222222218</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="I89" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+      <c r="I89" s="2">
+        <v>0.78650462962962964</v>
+      </c>
+      <c r="J89" s="2">
+        <v>0.78674768518518523</v>
+      </c>
+      <c r="K89" s="2">
+        <v>0.78901620370370373</v>
+      </c>
+      <c r="L89" s="2">
+        <v>0.78914351851851849</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B90" s="1">
-        <v>260811</v>
+        <v>260814</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>5</v>
@@ -4352,19 +4695,28 @@
         <v>108</v>
       </c>
       <c r="F90" s="2">
-        <v>0.78597222222222218</v>
+        <v>0.62765046296296301</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>125</v>
+        <v>229</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="I90" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+        <v>236</v>
+      </c>
+      <c r="I90" s="2">
+        <v>0.6283333333333333</v>
+      </c>
+      <c r="J90" s="2">
+        <v>0.62987268518518513</v>
+      </c>
+      <c r="K90" s="2">
+        <v>0.62988425925925928</v>
+      </c>
+      <c r="L90" s="2">
+        <v>0.63231481481481477</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>12</v>
       </c>
@@ -4372,28 +4724,37 @@
         <v>260814</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F91" s="2">
-        <v>0.62765046296296301</v>
+        <v>0.6489583333333333</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="I91" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+      <c r="I91" s="2">
+        <v>0.64952546296296299</v>
+      </c>
+      <c r="J91" s="2">
+        <v>0.65190972222222221</v>
+      </c>
+      <c r="K91" s="2">
+        <v>0.65192129629629625</v>
+      </c>
+      <c r="L91" s="2">
+        <v>0.65369212962962964</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>12</v>
       </c>
@@ -4401,28 +4762,37 @@
         <v>260814</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D92" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F92" s="2">
-        <v>0.6489583333333333</v>
+        <v>0.66555555555555557</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="I92" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+        <v>238</v>
+      </c>
+      <c r="I92" s="2">
+        <v>0.66630787037037043</v>
+      </c>
+      <c r="J92" s="2">
+        <v>0.66718750000000004</v>
+      </c>
+      <c r="K92" s="2">
+        <v>0.66888888888888887</v>
+      </c>
+      <c r="L92" s="2">
+        <v>0.67035879629629624</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>12</v>
       </c>
@@ -4430,28 +4800,37 @@
         <v>260814</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F93" s="2">
-        <v>0.66555555555555557</v>
+        <v>0.68576388888888884</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="I93" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+      <c r="I93" s="2">
+        <v>0.68636574074074075</v>
+      </c>
+      <c r="J93" s="2">
+        <v>0.68774305555555559</v>
+      </c>
+      <c r="K93" s="2">
+        <v>0.68989583333333337</v>
+      </c>
+      <c r="L93" s="2">
+        <v>0.69079861111111107</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>12</v>
       </c>
@@ -4459,28 +4838,37 @@
         <v>260814</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F94" s="2">
-        <v>0.68576388888888884</v>
+        <v>0.70138888888888884</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="I94" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+        <v>240</v>
+      </c>
+      <c r="I94" s="2">
+        <v>0.70192129629629629</v>
+      </c>
+      <c r="J94" s="2">
+        <v>0.70225694444444442</v>
+      </c>
+      <c r="K94" s="2">
+        <v>0.70424768518518521</v>
+      </c>
+      <c r="L94" s="2">
+        <v>0.70450231481481485</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>12</v>
       </c>
@@ -4488,28 +4876,37 @@
         <v>260814</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F95" s="2">
-        <v>0.70138888888888884</v>
+        <v>0.7149537037037037</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="I95" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+      <c r="I95" s="2">
+        <v>0.71542824074074074</v>
+      </c>
+      <c r="J95" s="2">
+        <v>0.71607638888888892</v>
+      </c>
+      <c r="K95" s="2">
+        <v>0.71726851851851847</v>
+      </c>
+      <c r="L95" s="2">
+        <v>0.71762731481481479</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>12</v>
       </c>
@@ -4517,51 +4914,78 @@
         <v>260814</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F96" s="2">
-        <v>0.7149537037037037</v>
+        <v>0.73736111111111113</v>
       </c>
       <c r="G96" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="I96" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+        <v>244</v>
+      </c>
+      <c r="I96" s="2">
+        <v>0.73811342592592588</v>
+      </c>
+      <c r="J96" s="2">
+        <v>0.73835648148148147</v>
+      </c>
+      <c r="K96" s="2">
+        <v>0.73974537037037036</v>
+      </c>
+      <c r="L96" s="2">
+        <v>0.73995370370370372</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B97" s="1">
-        <v>260814</v>
+        <v>260828</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="F97" s="2">
-        <v>0.73736111111111113</v>
-      </c>
-      <c r="I97" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0.60340277777777773</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H97" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="I97" s="2">
+        <v>0.60619212962962965</v>
+      </c>
+      <c r="J97" s="2">
+        <v>0.60638888888888887</v>
+      </c>
+      <c r="K97" s="2">
+        <v>0.60784722222222221</v>
+      </c>
+      <c r="L97" s="2">
+        <v>0.60793981481481485</v>
+      </c>
+      <c r="O97" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>13</v>
       </c>
@@ -4569,22 +4993,37 @@
         <v>260828</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D98" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F98" s="2">
-        <v>0.60340277777777773</v>
-      </c>
-      <c r="I98" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0.6134722222222222</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H98" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="I98" s="2">
+        <v>0.61561342592592594</v>
+      </c>
+      <c r="J98" s="2">
+        <v>0.61578703703703708</v>
+      </c>
+      <c r="K98" s="2">
+        <v>0.62050925925925926</v>
+      </c>
+      <c r="L98" s="2">
+        <v>0.62064814814814817</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>13</v>
       </c>
@@ -4592,22 +5031,37 @@
         <v>260828</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F99" s="2">
-        <v>0.6134722222222222</v>
-      </c>
-      <c r="I99" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0.63249999999999995</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H99" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="I99" s="2">
+        <v>0.63511574074074073</v>
+      </c>
+      <c r="J99" s="2">
+        <v>0.63525462962962964</v>
+      </c>
+      <c r="K99" s="2">
+        <v>0.638275462962963</v>
+      </c>
+      <c r="L99" s="2">
+        <v>0.63842592592592595</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>13</v>
       </c>
@@ -4615,22 +5069,37 @@
         <v>260828</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F100" s="2">
-        <v>0.63249999999999995</v>
-      </c>
-      <c r="I100" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0.64784722222222224</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H100" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="I100" s="2">
+        <v>0.64975694444444443</v>
+      </c>
+      <c r="J100" s="2">
+        <v>0.6498842592592593</v>
+      </c>
+      <c r="K100" s="2">
+        <v>0.6529166666666667</v>
+      </c>
+      <c r="L100" s="2">
+        <v>0.65300925925925923</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>13</v>
       </c>
@@ -4638,22 +5107,40 @@
         <v>260828</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D101" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F101" s="2">
-        <v>0.64784722222222224</v>
-      </c>
-      <c r="I101" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0.65902777777777777</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="I101" s="2">
+        <v>0.66045138888888888</v>
+      </c>
+      <c r="J101" s="2">
+        <v>0.66061342592592598</v>
+      </c>
+      <c r="K101" s="2">
+        <v>0.66343750000000001</v>
+      </c>
+      <c r="L101" s="2">
+        <v>0.66350694444444447</v>
+      </c>
+      <c r="O101" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>13</v>
       </c>
@@ -4661,22 +5148,37 @@
         <v>260828</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D102" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F102" s="2">
-        <v>0.65902777777777777</v>
-      </c>
-      <c r="I102" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0.67945601851851856</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H102" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="I102" s="2">
+        <v>0.68041666666666667</v>
+      </c>
+      <c r="J102" s="2">
+        <v>0.6806712962962963</v>
+      </c>
+      <c r="K102" s="2">
+        <v>0.68125000000000002</v>
+      </c>
+      <c r="L102" s="2">
+        <v>0.68157407407407411</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>13</v>
       </c>
@@ -4684,42 +5186,34 @@
         <v>260828</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F103" s="2">
-        <v>0.67945601851851856</v>
-      </c>
-      <c r="I103" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A104" s="1">
-        <v>13</v>
-      </c>
-      <c r="B104" s="1">
-        <v>260828</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D104" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E104" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="F104" s="2">
         <v>0.69167824074074069</v>
       </c>
-      <c r="I104" s="1" t="s">
-        <v>205</v>
+      <c r="G103" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="H103" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="I103" s="2">
+        <v>0.69403935185185184</v>
+      </c>
+      <c r="J103" s="2">
+        <v>0.69447916666666665</v>
+      </c>
+      <c r="K103" s="2">
+        <v>0.69465277777777779</v>
+      </c>
+      <c r="L103" s="2">
+        <v>0.69498842592592591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>